<commit_message>
feat: prompt rows with any number of images, row add/delete, bulk image rules
Excel/CSV rows are prompts in order; the anh column lists several images
(; separated) resolved against the folder's image library, and missing
rows are added. Start checks the image count per mode (frame: exactly 1,
reference: 1–10).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/mau-nhap-theo-ten-anh.xlsx
+++ b/samples/mau-nhap-theo-ten-anh.xlsx
@@ -90,9 +90,7 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -476,7 +474,7 @@
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>anh</t>
@@ -571,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -580,73 +578,80 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>Mẫu nhập theo TÊN ẢNH</t>
+          <t>Mẫu: mỗi prompt một ảnh</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Cột anh = tên file ảnh trong folder ảnh (có hoặc không có đuôi, không phân biệt hoa thường). Thứ tự dòng không quan trọng.</t>
-        </is>
-      </c>
+      <c r="A2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ô nền vàng ở sheet đầu tiên là chỗ để sửa. Các dòng có sẵn là ví dụ: xoá đi rồi nhập dữ liệu của bạn.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Ô nền vàng ở sheet đầu tiên là chỗ để sửa. Các dòng có sẵn là ví dụ: xoá đi rồi nhập dữ liệu của bạn.</t>
+          <t>Tool chỉ đọc SHEET ĐẦU TIÊN. Giữ nguyên dòng tiêu đề (dòng 1); không cần đủ mọi cột.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Tool chỉ đọc SHEET ĐẦU TIÊN. Giữ nguyên dòng tiêu đề (dòng 1); không cần đủ mọi cột.</t>
+          <t>Mỗi dòng dữ liệu là MỘT PROMPT, theo thứ tự: dòng 2 trong Excel = prompt 1, dòng 3 = prompt 2… Thiếu dòng trong tool thì tool tự thêm.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>prompt — mô tả chuyển động/cảnh cho Veo (nên viết tiếng Anh). Ô trống = dùng Prompt chung trong tool.</t>
+          <t>anh — tên ảnh trong folder ảnh của dự án (có hoặc không có đuôi). Nhiều ảnh thì cách nhau bằng dấu ; (ví dụ: a.png; b.png). Ô trống = giữ ảnh đang có của prompt đó.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>text — chữ hiện trên video ở bước 2 Hậu kỳ. Ô trống = giữ text đang có.</t>
+          <t>Chế độ 'Ảnh làm khung đầu' dùng đúng 1 ảnh mỗi prompt; chế độ 'Ảnh tham chiếu' dùng 1–10 ảnh mỗi prompt.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>nhac — tên file nhạc nằm trong folder nhạc đã chọn ở bước 2 (ví dụ nhac-1.mp3). Ô trống = nhạc theo chế độ chung.</t>
+          <t>prompt — mô tả cho Veo (nên viết tiếng Anh). Ô trống = dùng Prompt chung trong tool.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Ô trống không bao giờ xoá dữ liệu đang có trong tool.</t>
+          <t>text — chữ hiện trên video ở bước 2 Hậu kỳ. Ô trống = giữ text đang có.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Cách nhập: trong tool bấm 'Nhập Excel/CSV' (có ở cả bước 1 và bước 2) rồi chọn file này.</t>
+          <t>nhac — tên file nhạc trong folder nhạc đã chọn ở bước 2 (ví dụ nhac-1.mp3). Ô trống = nhạc theo chế độ chung.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Nếu lưu dạng CSV: trong Excel chọn 'CSV UTF-8 (Comma delimited)' để giữ dấu tiếng Việt.</t>
+          <t>Ô trống không bao giờ xoá dữ liệu đang có. Tên ảnh không tìm thấy sẽ được báo lại.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Cách nhập: trong tool bấm 'Nhập Excel/CSV' (có ở cả bước 1 và bước 2) rồi chọn file này. CSV thì lưu dạng 'CSV UTF-8'.</t>
         </is>
       </c>
     </row>

</xml_diff>